<commit_message>
sample_data: drop plug threshold, always plug Cassa to balance SP
Removed the |gap| < 5 guard from build_sample_data.py: the script now
always closes the residual SP gap into "Cassa e disponibilità" so all
years balance exactly.

Plug applied:
- Tier 1 / Y0: gap = 0 (no-op).
- Tier 2 / Y-1: Cassa 162 -> 197 (+35).
- Tier 2 / Y0:  Cassa 180 -> 217 (+37).

Post-plug SP sum = 0 for Tier 1 Y0, Tier 2 Y-1, Tier 2 Y0.

https://claude.ai/code/session_01NBSvkpKwm8FK7SzrAxk78f
</commit_message>
<xml_diff>
--- a/projection_library_kernel_v1.1/projection_library/sample_data/tier2_industrial_clean.xlsx
+++ b/projection_library_kernel_v1.1/projection_library/sample_data/tier2_industrial_clean.xlsx
@@ -630,10 +630,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>162</v>
+        <v>197</v>
       </c>
       <c r="D12" t="n">
-        <v>180</v>
+        <v>217</v>
       </c>
     </row>
     <row r="13">

</xml_diff>